<commit_message>
Add per-call telemetry to the comparison workbook
docs/accuracy.txt asks for tokens "per page ... on a call basis", which
the per-document rollup does not answer. The new Calls sheet is one row
per API request: stage, model, page window, tokens, latency and cost,
split input and output.

Per-page figures divide by the pages that call actually carried, read
from its own `pages` window, not by the document total — a layout call
reading 5 header pages and an extraction call reading 50 are not the
same unit. A text-source call carries `text` rather than a range and
reports no page count, which is not the same as zero.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/qa_results_new/v1_20260807_202952.xlsx
+++ b/qa_results_new/v1_20260807_202952.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="61" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-07 20:51:22</t>
+          <t>2026-08-07 20:57:16</t>
         </is>
       </c>
     </row>
@@ -478,7 +478,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
@@ -500,7 +500,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6">
@@ -510,7 +510,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7">
@@ -520,7 +520,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>93.8</v>
+        <v>88.90000000000001</v>
       </c>
     </row>
     <row r="8">
@@ -530,7 +530,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>245</v>
+        <v>268</v>
       </c>
     </row>
     <row r="9">
@@ -540,7 +540,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>210</v>
+        <v>232</v>
       </c>
     </row>
     <row r="10">
@@ -550,7 +550,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>85.7</v>
+        <v>86.59999999999999</v>
       </c>
     </row>
     <row r="11"/>
@@ -712,6 +712,78 @@
         <v>0</v>
       </c>
       <c r="J16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>18-19 GL Loss Run - United Specialty.pdf</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>openai/gpt-5.6-luna</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" t="n">
+        <v>100</v>
+      </c>
+      <c r="G17" t="n">
+        <v>23</v>
+      </c>
+      <c r="H17" t="n">
+        <v>22</v>
+      </c>
+      <c r="I17" t="n">
+        <v>95.7</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>18-19 XS Loss Runs - AIG.pdf</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>1</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>openai/gpt-5.6-luna</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" t="n">
         <v>0</v>
       </c>
     </row>
@@ -780,13 +852,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D3" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4">
@@ -796,13 +868,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D4" t="n">
-        <v>46.7</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5">
@@ -812,45 +884,45 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D5" t="n">
-        <v>60</v>
+        <v>62.5</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Claimant Name</t>
+          <t>Line of Business</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C6" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D6" t="n">
-        <v>76.90000000000001</v>
+        <v>75</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Line of Business</t>
+          <t>Claimant Name</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C7" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D7" t="n">
-        <v>80</v>
+        <v>78.59999999999999</v>
       </c>
     </row>
     <row r="8">
@@ -860,13 +932,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C8" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D8" t="n">
-        <v>80</v>
+        <v>81.2</v>
       </c>
     </row>
     <row r="9">
@@ -876,10 +948,10 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C9" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D9" t="n">
         <v>100</v>
@@ -892,10 +964,10 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C10" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D10" t="n">
         <v>100</v>
@@ -908,10 +980,10 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C11" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D11" t="n">
         <v>100</v>
@@ -924,10 +996,10 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C12" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D12" t="n">
         <v>100</v>
@@ -940,10 +1012,10 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D13" t="n">
         <v>100</v>
@@ -956,10 +1028,10 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C14" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D14" t="n">
         <v>100</v>
@@ -972,10 +1044,10 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D15" t="n">
         <v>100</v>
@@ -988,10 +1060,10 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C16" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D16" t="n">
         <v>100</v>
@@ -1004,10 +1076,10 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C17" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D17" t="n">
         <v>100</v>
@@ -1020,10 +1092,10 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C18" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D18" t="n">
         <v>100</v>
@@ -1036,10 +1108,10 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C19" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D19" t="n">
         <v>100</v>
@@ -1052,10 +1124,10 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D20" t="n">
         <v>100</v>
@@ -1068,10 +1140,10 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C21" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D21" t="n">
         <v>100</v>
@@ -1084,10 +1156,10 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C22" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D22" t="n">
         <v>100</v>
@@ -1100,10 +1172,10 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C23" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D23" t="n">
         <v>100</v>
@@ -1116,10 +1188,10 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C24" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D24" t="n">
         <v>100</v>
@@ -1132,10 +1204,10 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C25" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D25" t="n">
         <v>100</v>
@@ -1242,28 +1314,28 @@
         </is>
       </c>
       <c r="D2" t="n">
+        <v>18</v>
+      </c>
+      <c r="E2" t="n">
         <v>16</v>
       </c>
-      <c r="E2" t="n">
-        <v>15</v>
-      </c>
       <c r="F2" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G2" t="n">
-        <v>245</v>
+        <v>268</v>
       </c>
       <c r="H2" t="n">
-        <v>257</v>
+        <v>280</v>
       </c>
       <c r="I2" t="n">
-        <v>85.7</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="J2" t="n">
-        <v>81.7</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="K2" t="n">
-        <v>4</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="3">
@@ -1283,25 +1355,25 @@
         </is>
       </c>
       <c r="D3" t="n">
+        <v>18</v>
+      </c>
+      <c r="E3" t="n">
         <v>16</v>
       </c>
-      <c r="E3" t="n">
-        <v>15</v>
-      </c>
       <c r="F3" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G3" t="n">
-        <v>245</v>
+        <v>268</v>
       </c>
       <c r="H3" t="n">
-        <v>245</v>
+        <v>268</v>
       </c>
       <c r="I3" t="n">
-        <v>85.7</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="J3" t="n">
-        <v>85.7</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="K3" t="n">
         <v>0</v>
@@ -1324,25 +1396,25 @@
         </is>
       </c>
       <c r="D4" t="n">
+        <v>18</v>
+      </c>
+      <c r="E4" t="n">
         <v>16</v>
       </c>
-      <c r="E4" t="n">
-        <v>15</v>
-      </c>
       <c r="F4" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G4" t="n">
-        <v>245</v>
+        <v>268</v>
       </c>
       <c r="H4" t="n">
-        <v>245</v>
+        <v>268</v>
       </c>
       <c r="I4" t="n">
-        <v>85.7</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="J4" t="n">
-        <v>85.7</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="K4" t="n">
         <v>0</v>
@@ -1365,25 +1437,25 @@
         </is>
       </c>
       <c r="D5" t="n">
+        <v>18</v>
+      </c>
+      <c r="E5" t="n">
         <v>16</v>
       </c>
-      <c r="E5" t="n">
-        <v>15</v>
-      </c>
       <c r="F5" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G5" t="n">
-        <v>245</v>
+        <v>268</v>
       </c>
       <c r="H5" t="n">
-        <v>245</v>
+        <v>268</v>
       </c>
       <c r="I5" t="n">
-        <v>85.7</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="J5" t="n">
-        <v>85.7</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="K5" t="n">
         <v>0</v>
@@ -1406,25 +1478,25 @@
         </is>
       </c>
       <c r="D6" t="n">
+        <v>18</v>
+      </c>
+      <c r="E6" t="n">
         <v>16</v>
       </c>
-      <c r="E6" t="n">
-        <v>15</v>
-      </c>
       <c r="F6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G6" t="n">
-        <v>245</v>
+        <v>268</v>
       </c>
       <c r="H6" t="n">
-        <v>245</v>
+        <v>268</v>
       </c>
       <c r="I6" t="n">
-        <v>85.7</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="J6" t="n">
-        <v>85.7</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="K6" t="n">
         <v>0</v>
@@ -1447,28 +1519,28 @@
         </is>
       </c>
       <c r="D7" t="n">
+        <v>18</v>
+      </c>
+      <c r="E7" t="n">
         <v>16</v>
       </c>
-      <c r="E7" t="n">
-        <v>15</v>
-      </c>
       <c r="F7" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G7" t="n">
-        <v>245</v>
+        <v>268</v>
       </c>
       <c r="H7" t="n">
-        <v>245</v>
+        <v>268</v>
       </c>
       <c r="I7" t="n">
-        <v>85.7</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="J7" t="n">
-        <v>84.90000000000001</v>
+        <v>85.8</v>
       </c>
       <c r="K7" t="n">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="8"/>
@@ -1567,7 +1639,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V15"/>
+  <dimension ref="A1:V23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1932,281 +2004,271 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5"/>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>5185622e</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>196521831d58</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2026-08-07 20:51:24</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>18-19 GL Loss Run - United Specialty.pdf</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>openai/gpt-5.6-luna</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>max</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" t="n">
+        <v>1</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" t="n">
+        <v>100</v>
+      </c>
+      <c r="N5" t="n">
+        <v>100</v>
+      </c>
+      <c r="O5" t="n">
+        <v>23</v>
+      </c>
+      <c r="P5" t="n">
+        <v>22</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>95.7</v>
+      </c>
+      <c r="R5" t="n">
+        <v>95.7</v>
+      </c>
+      <c r="S5" t="n">
+        <v>95.7</v>
+      </c>
+      <c r="T5" t="n">
+        <v>0</v>
+      </c>
+      <c r="U5" t="n">
+        <v>0</v>
+      </c>
+    </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>5185622e</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>3e0fb97b3ce7</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2026-08-07 20:52:40</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>18-19 XS Loss Runs - AIG.pdf</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>openai/gpt-5.6-luna</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>max</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I6" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
+        <v>1</v>
+      </c>
+      <c r="L6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7"/>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>run_id</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>document</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>stage</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>model</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>provider</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>label</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>pages</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>attempt</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>effort</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>response_id</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>latency_s</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>poll_count</t>
         </is>
       </c>
-      <c r="N6" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>input_tokens</t>
         </is>
       </c>
-      <c r="O6" s="2" t="inlineStr">
+      <c r="O8" s="2" t="inlineStr">
         <is>
           <t>output_tokens</t>
         </is>
       </c>
-      <c r="P6" s="2" t="inlineStr">
+      <c r="P8" s="2" t="inlineStr">
         <is>
           <t>total_tokens</t>
         </is>
       </c>
-      <c r="Q6" s="2" t="inlineStr">
+      <c r="Q8" s="2" t="inlineStr">
         <is>
           <t>cost_input_usd</t>
         </is>
       </c>
-      <c r="R6" s="2" t="inlineStr">
+      <c r="R8" s="2" t="inlineStr">
         <is>
           <t>cost_output_usd</t>
         </is>
       </c>
-      <c r="S6" s="2" t="inlineStr">
+      <c r="S8" s="2" t="inlineStr">
         <is>
           <t>cost_total_usd</t>
         </is>
       </c>
-      <c r="T6" s="2" t="inlineStr">
+      <c r="T8" s="2" t="inlineStr">
         <is>
           <t>usage_missing</t>
         </is>
       </c>
-      <c r="U6" s="2" t="inlineStr">
+      <c r="U8" s="2" t="inlineStr">
         <is>
           <t>error_code</t>
         </is>
       </c>
-      <c r="V6" s="2" t="inlineStr">
+      <c r="V8" s="2" t="inlineStr">
         <is>
           <t>error_message</t>
         </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>40f183e1a55f</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>05.09.2020 to 6-30-2022- GL only Policy Loss Run Report.pdf</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>layout</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>openai/gpt-5.6-luna</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>openai</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>layout discovery</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>1-5</t>
-        </is>
-      </c>
-      <c r="H7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>resp_0a4ea48cef7acdd3006a75f2ec13e4819393d541a8699901d6</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>completed</t>
-        </is>
-      </c>
-      <c r="L7" t="n">
-        <v>19.07</v>
-      </c>
-      <c r="M7" t="n">
-        <v>4</v>
-      </c>
-      <c r="N7" t="n">
-        <v>20226</v>
-      </c>
-      <c r="O7" t="n">
-        <v>1349</v>
-      </c>
-      <c r="P7" t="n">
-        <v>21575</v>
-      </c>
-      <c r="Q7" t="n">
-        <v>0.004045</v>
-      </c>
-      <c r="R7" t="n">
-        <v>0.001079</v>
-      </c>
-      <c r="S7" t="n">
-        <v>0.005124</v>
-      </c>
-      <c r="T7" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>40f183e1a55f</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>05.09.2020 to 6-30-2022- GL only Policy Loss Run Report.pdf</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>extract</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>openai/gpt-5.6-luna</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>openai</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>chunk 1/1</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>1-10</t>
-        </is>
-      </c>
-      <c r="H8" t="n">
-        <v>1</v>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>max</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>resp_08a100fa287cdf15006a75f2fbd2708190bd7a78a62d98e308</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>completed</t>
-        </is>
-      </c>
-      <c r="L8" t="n">
-        <v>18.55</v>
-      </c>
-      <c r="M8" t="n">
-        <v>4</v>
-      </c>
-      <c r="N8" t="n">
-        <v>35968</v>
-      </c>
-      <c r="O8" t="n">
-        <v>21734</v>
-      </c>
-      <c r="P8" t="n">
-        <v>57702</v>
-      </c>
-      <c r="Q8" t="n">
-        <v>0.007194</v>
-      </c>
-      <c r="R8" t="n">
-        <v>0.017387</v>
-      </c>
-      <c r="S8" t="n">
-        <v>0.024581</v>
-      </c>
-      <c r="T8" t="b">
-        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -2222,7 +2284,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>qa</t>
+          <t>layout</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -2237,12 +2299,12 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>chunk 1/1</t>
+          <t>layout discovery</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>1-10</t>
+          <t>1-5</t>
         </is>
       </c>
       <c r="H9" t="n">
@@ -2250,12 +2312,12 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>max</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>resp_03817eba275b785f006a75f5e9e57481968eb800249d5c5530</t>
+          <t>resp_0a4ea48cef7acdd3006a75f2ec13e4819393d541a8699901d6</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -2264,28 +2326,28 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>68.41</v>
+        <v>19.07</v>
       </c>
       <c r="M9" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="N9" t="n">
-        <v>38119</v>
+        <v>20226</v>
       </c>
       <c r="O9" t="n">
-        <v>7415</v>
+        <v>1349</v>
       </c>
       <c r="P9" t="n">
-        <v>45534</v>
+        <v>21575</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.007624</v>
+        <v>0.004045</v>
       </c>
       <c r="R9" t="n">
-        <v>0.005932</v>
+        <v>0.001079</v>
       </c>
       <c r="S9" t="n">
-        <v>0.013556</v>
+        <v>0.005124</v>
       </c>
       <c r="T9" t="b">
         <v>0</v>
@@ -2294,17 +2356,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1759b6f93b6b</t>
+          <t>40f183e1a55f</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>16-18 GL Loss Runs - Twenty Mile Acceptance.pdf</t>
+          <t>05.09.2020 to 6-30-2022- GL only Policy Loss Run Report.pdf</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>layout</t>
+          <t>extract</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -2319,12 +2381,12 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>layout discovery</t>
+          <t>chunk 1/1</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>1-2</t>
+          <t>1-10</t>
         </is>
       </c>
       <c r="H10" t="n">
@@ -2332,12 +2394,12 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>max</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>resp_00fb79eac91891a0006a75f62f921c8197be64661c1c6f20f0</t>
+          <t>resp_08a100fa287cdf15006a75f2fbd2708190bd7a78a62d98e308</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -2346,28 +2408,28 @@
         </is>
       </c>
       <c r="L10" t="n">
-        <v>19.56</v>
+        <v>18.55</v>
       </c>
       <c r="M10" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N10" t="n">
-        <v>12042</v>
+        <v>35968</v>
       </c>
       <c r="O10" t="n">
-        <v>1452</v>
+        <v>21734</v>
       </c>
       <c r="P10" t="n">
-        <v>13494</v>
+        <v>57702</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.002408</v>
+        <v>0.007194</v>
       </c>
       <c r="R10" t="n">
-        <v>0.001162</v>
+        <v>0.017387</v>
       </c>
       <c r="S10" t="n">
-        <v>0.00357</v>
+        <v>0.024581</v>
       </c>
       <c r="T10" t="b">
         <v>0</v>
@@ -2376,17 +2438,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1759b6f93b6b</t>
+          <t>40f183e1a55f</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>16-18 GL Loss Runs - Twenty Mile Acceptance.pdf</t>
+          <t>05.09.2020 to 6-30-2022- GL only Policy Loss Run Report.pdf</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>extract</t>
+          <t>qa</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -2406,7 +2468,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>1-2</t>
+          <t>1-10</t>
         </is>
       </c>
       <c r="H11" t="n">
@@ -2419,7 +2481,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>resp_0752f25ff5cc747d006a75f642fe908196bf92abb84f96a388</t>
+          <t>resp_03817eba275b785f006a75f5e9e57481968eb800249d5c5530</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -2428,28 +2490,28 @@
         </is>
       </c>
       <c r="L11" t="n">
-        <v>44.8</v>
+        <v>68.41</v>
       </c>
       <c r="M11" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="N11" t="n">
-        <v>12490</v>
+        <v>38119</v>
       </c>
       <c r="O11" t="n">
-        <v>5763</v>
+        <v>7415</v>
       </c>
       <c r="P11" t="n">
-        <v>18253</v>
+        <v>45534</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.002498</v>
+        <v>0.007624</v>
       </c>
       <c r="R11" t="n">
-        <v>0.00461</v>
+        <v>0.005932</v>
       </c>
       <c r="S11" t="n">
-        <v>0.007108</v>
+        <v>0.013556</v>
       </c>
       <c r="T11" t="b">
         <v>0</v>
@@ -2468,7 +2530,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>qa</t>
+          <t>layout</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -2483,7 +2545,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>chunk 1/1</t>
+          <t>layout discovery</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -2496,12 +2558,12 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>max</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>resp_01d001704000e301006a75f66f9edc81958828c4f26587423d</t>
+          <t>resp_00fb79eac91891a0006a75f62f921c8197be64661c1c6f20f0</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -2510,28 +2572,28 @@
         </is>
       </c>
       <c r="L12" t="n">
-        <v>59.56</v>
+        <v>19.56</v>
       </c>
       <c r="M12" t="n">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="N12" t="n">
-        <v>13093</v>
+        <v>12042</v>
       </c>
       <c r="O12" t="n">
-        <v>6964</v>
+        <v>1452</v>
       </c>
       <c r="P12" t="n">
-        <v>20057</v>
+        <v>13494</v>
       </c>
       <c r="Q12" t="n">
-        <v>0.002619</v>
+        <v>0.002408</v>
       </c>
       <c r="R12" t="n">
-        <v>0.005571</v>
+        <v>0.001162</v>
       </c>
       <c r="S12" t="n">
-        <v>0.008189999999999999</v>
+        <v>0.00357</v>
       </c>
       <c r="T12" t="b">
         <v>0</v>
@@ -2540,17 +2602,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ccf6dacf0369</t>
+          <t>1759b6f93b6b</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>17-18 XS Loss Runs - AIG.pdf</t>
+          <t>16-18 GL Loss Runs - Twenty Mile Acceptance.pdf</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>layout</t>
+          <t>extract</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -2565,7 +2627,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>layout discovery</t>
+          <t>chunk 1/1</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -2578,12 +2640,12 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>max</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>resp_08e02d502f20a249006a75f6ad54bc819597d747c0721b717d</t>
+          <t>resp_0752f25ff5cc747d006a75f642fe908196bf92abb84f96a388</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -2592,28 +2654,28 @@
         </is>
       </c>
       <c r="L13" t="n">
-        <v>24</v>
+        <v>44.8</v>
       </c>
       <c r="M13" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="N13" t="n">
-        <v>9668</v>
+        <v>12490</v>
       </c>
       <c r="O13" t="n">
-        <v>1895</v>
+        <v>5763</v>
       </c>
       <c r="P13" t="n">
-        <v>11563</v>
+        <v>18253</v>
       </c>
       <c r="Q13" t="n">
-        <v>0.001934</v>
+        <v>0.002498</v>
       </c>
       <c r="R13" t="n">
-        <v>0.001516</v>
+        <v>0.00461</v>
       </c>
       <c r="S13" t="n">
-        <v>0.00345</v>
+        <v>0.007108</v>
       </c>
       <c r="T13" t="b">
         <v>0</v>
@@ -2622,17 +2684,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ccf6dacf0369</t>
+          <t>1759b6f93b6b</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>17-18 XS Loss Runs - AIG.pdf</t>
+          <t>16-18 GL Loss Runs - Twenty Mile Acceptance.pdf</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>extract</t>
+          <t>qa</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -2665,7 +2727,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>resp_03005e22cdeeb03c006a75f6c5118c8195a40866eb7979f3d3</t>
+          <t>resp_01d001704000e301006a75f66f9edc81958828c4f26587423d</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -2674,28 +2736,28 @@
         </is>
       </c>
       <c r="L14" t="n">
-        <v>103.07</v>
+        <v>59.56</v>
       </c>
       <c r="M14" t="n">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="N14" t="n">
-        <v>10034</v>
+        <v>13093</v>
       </c>
       <c r="O14" t="n">
-        <v>13255</v>
+        <v>6964</v>
       </c>
       <c r="P14" t="n">
-        <v>23289</v>
+        <v>20057</v>
       </c>
       <c r="Q14" t="n">
-        <v>0.002007</v>
+        <v>0.002619</v>
       </c>
       <c r="R14" t="n">
-        <v>0.010604</v>
+        <v>0.005571</v>
       </c>
       <c r="S14" t="n">
-        <v>0.012611</v>
+        <v>0.008189999999999999</v>
       </c>
       <c r="T14" t="b">
         <v>0</v>
@@ -2714,7 +2776,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>qa</t>
+          <t>layout</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -2729,7 +2791,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>chunk 1/1</t>
+          <t>layout discovery</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -2742,44 +2804,700 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>resp_08e02d502f20a249006a75f6ad54bc819597d747c0721b717d</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="L15" t="n">
+        <v>24</v>
+      </c>
+      <c r="M15" t="n">
+        <v>6</v>
+      </c>
+      <c r="N15" t="n">
+        <v>9668</v>
+      </c>
+      <c r="O15" t="n">
+        <v>1895</v>
+      </c>
+      <c r="P15" t="n">
+        <v>11563</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>0.001934</v>
+      </c>
+      <c r="R15" t="n">
+        <v>0.001516</v>
+      </c>
+      <c r="S15" t="n">
+        <v>0.00345</v>
+      </c>
+      <c r="T15" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>ccf6dacf0369</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>17-18 XS Loss Runs - AIG.pdf</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>extract</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>openai/gpt-5.6-luna</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>openai</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>chunk 1/1</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H16" t="n">
+        <v>1</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
           <t>max</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>resp_03005e22cdeeb03c006a75f6c5118c8195a40866eb7979f3d3</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="L16" t="n">
+        <v>103.07</v>
+      </c>
+      <c r="M16" t="n">
+        <v>26</v>
+      </c>
+      <c r="N16" t="n">
+        <v>10034</v>
+      </c>
+      <c r="O16" t="n">
+        <v>13255</v>
+      </c>
+      <c r="P16" t="n">
+        <v>23289</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>0.002007</v>
+      </c>
+      <c r="R16" t="n">
+        <v>0.010604</v>
+      </c>
+      <c r="S16" t="n">
+        <v>0.012611</v>
+      </c>
+      <c r="T16" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>ccf6dacf0369</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>17-18 XS Loss Runs - AIG.pdf</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>qa</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>openai/gpt-5.6-luna</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>openai</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>chunk 1/1</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>max</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
         <is>
           <t>resp_0a2bcc8f490832f6006a75f72c17dc8195ab8e88d1bb16c34b</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="K17" t="inlineStr">
         <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="L15" t="n">
+      <c r="L17" t="n">
         <v>138.92</v>
       </c>
-      <c r="M15" t="n">
+      <c r="M17" t="n">
         <v>37</v>
       </c>
-      <c r="N15" t="n">
+      <c r="N17" t="n">
         <v>10309</v>
       </c>
-      <c r="O15" t="n">
+      <c r="O17" t="n">
         <v>23380</v>
       </c>
-      <c r="P15" t="n">
+      <c r="P17" t="n">
         <v>33689</v>
       </c>
-      <c r="Q15" t="n">
+      <c r="Q17" t="n">
         <v>0.002062</v>
       </c>
-      <c r="R15" t="n">
+      <c r="R17" t="n">
         <v>0.018704</v>
       </c>
-      <c r="S15" t="n">
+      <c r="S17" t="n">
         <v>0.020766</v>
       </c>
-      <c r="T15" t="b">
+      <c r="T17" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>196521831d58</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>18-19 GL Loss Run - United Specialty.pdf</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>layout</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>openai/gpt-5.6-luna</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>openai</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>layout discovery</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H18" t="n">
+        <v>1</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>resp_07524a2d2b102f7f006a75f7f4ca1881909daf67de0228efe6</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="L18" t="n">
+        <v>16.31</v>
+      </c>
+      <c r="M18" t="n">
+        <v>4</v>
+      </c>
+      <c r="N18" t="n">
+        <v>8261</v>
+      </c>
+      <c r="O18" t="n">
+        <v>1393</v>
+      </c>
+      <c r="P18" t="n">
+        <v>9654</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>0.001652</v>
+      </c>
+      <c r="R18" t="n">
+        <v>0.001114</v>
+      </c>
+      <c r="S18" t="n">
+        <v>0.002767</v>
+      </c>
+      <c r="T18" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>196521831d58</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>18-19 GL Loss Run - United Specialty.pdf</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>extract</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>openai/gpt-5.6-luna</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>openai</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>chunk 1/1</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>max</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>resp_0ecd97c337817288006a75f804d5ac8190a98cec5129c5f380</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="L19" t="n">
+        <v>22.74</v>
+      </c>
+      <c r="M19" t="n">
+        <v>6</v>
+      </c>
+      <c r="N19" t="n">
+        <v>8651</v>
+      </c>
+      <c r="O19" t="n">
+        <v>2575</v>
+      </c>
+      <c r="P19" t="n">
+        <v>11226</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>0.00173</v>
+      </c>
+      <c r="R19" t="n">
+        <v>0.00206</v>
+      </c>
+      <c r="S19" t="n">
+        <v>0.00379</v>
+      </c>
+      <c r="T19" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>196521831d58</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>18-19 GL Loss Run - United Specialty.pdf</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>qa</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>openai/gpt-5.6-luna</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>openai</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>chunk 1/1</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H20" t="n">
+        <v>1</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>max</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>resp_04ffca1fcc2e0ecc006a75f81b8ea88193a1aa1ce03f5ac990</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="L20" t="n">
+        <v>34.13</v>
+      </c>
+      <c r="M20" t="n">
+        <v>9</v>
+      </c>
+      <c r="N20" t="n">
+        <v>8902</v>
+      </c>
+      <c r="O20" t="n">
+        <v>3536</v>
+      </c>
+      <c r="P20" t="n">
+        <v>12438</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>0.00178</v>
+      </c>
+      <c r="R20" t="n">
+        <v>0.002829</v>
+      </c>
+      <c r="S20" t="n">
+        <v>0.004609</v>
+      </c>
+      <c r="T20" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>3e0fb97b3ce7</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>18-19 XS Loss Runs - AIG.pdf</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>layout</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>openai/gpt-5.6-luna</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>openai</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>layout discovery</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H21" t="n">
+        <v>1</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>resp_029cf6536e8ff7b5006a75f84167c481949dd80cb7ea79b942</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="L21" t="n">
+        <v>23.57</v>
+      </c>
+      <c r="M21" t="n">
+        <v>6</v>
+      </c>
+      <c r="N21" t="n">
+        <v>7368</v>
+      </c>
+      <c r="O21" t="n">
+        <v>1851</v>
+      </c>
+      <c r="P21" t="n">
+        <v>9219</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>0.001474</v>
+      </c>
+      <c r="R21" t="n">
+        <v>0.001481</v>
+      </c>
+      <c r="S21" t="n">
+        <v>0.002954</v>
+      </c>
+      <c r="T21" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>3e0fb97b3ce7</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>18-19 XS Loss Runs - AIG.pdf</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>extract</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>openai/gpt-5.6-luna</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>openai</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>chunk 1/1</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H22" t="n">
+        <v>1</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>max</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>resp_0dbf9fdfbe24bcaf006a75f858be408196b5564146a5d5d081</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="L22" t="n">
+        <v>103.6</v>
+      </c>
+      <c r="M22" t="n">
+        <v>28</v>
+      </c>
+      <c r="N22" t="n">
+        <v>7683</v>
+      </c>
+      <c r="O22" t="n">
+        <v>13721</v>
+      </c>
+      <c r="P22" t="n">
+        <v>21404</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>0.001537</v>
+      </c>
+      <c r="R22" t="n">
+        <v>0.010977</v>
+      </c>
+      <c r="S22" t="n">
+        <v>0.012513</v>
+      </c>
+      <c r="T22" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>3e0fb97b3ce7</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>18-19 XS Loss Runs - AIG.pdf</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>qa</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>openai/gpt-5.6-luna</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>openai</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>chunk 1/1</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H23" t="n">
+        <v>1</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>max</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>resp_0c97261014dfacf8006a75f8c04fd88190addffbea021f4f99</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="L23" t="n">
+        <v>131.5</v>
+      </c>
+      <c r="M23" t="n">
+        <v>35</v>
+      </c>
+      <c r="N23" t="n">
+        <v>7968</v>
+      </c>
+      <c r="O23" t="n">
+        <v>18533</v>
+      </c>
+      <c r="P23" t="n">
+        <v>26501</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>0.001594</v>
+      </c>
+      <c r="R23" t="n">
+        <v>0.014826</v>
+      </c>
+      <c r="S23" t="n">
+        <v>0.01642</v>
+      </c>
+      <c r="T23" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Record the poll-loop telemetry blind spot as CHALLENGES #24
A document in the extended run took 91.6 minutes of wall clock containing
9.3 minutes of recorded API calls. The gap is sporadic — five of seven
documents show under a minute — but the ledger provably cannot see it:
_poll retries on httpx errors and on 503 without recording anything, so a
call row reports one latency however many silent retries happened inside.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/qa_results_new/v1_20260807_202952.xlsx
+++ b/qa_results_new/v1_20260807_202952.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J18"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="61" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-07 20:57:16</t>
+          <t>2026-08-07 22:28:56</t>
         </is>
       </c>
     </row>
@@ -478,7 +478,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4">
@@ -500,7 +500,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>18</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6">
@@ -510,7 +510,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7">
@@ -520,7 +520,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>88.90000000000001</v>
+        <v>43.6</v>
       </c>
     </row>
     <row r="8">
@@ -530,7 +530,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>268</v>
+        <v>287</v>
       </c>
     </row>
     <row r="9">
@@ -540,7 +540,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>232</v>
+        <v>244</v>
       </c>
     </row>
     <row r="10">
@@ -550,7 +550,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>86.59999999999999</v>
+        <v>85</v>
       </c>
     </row>
     <row r="11"/>
@@ -784,6 +784,42 @@
         <v>0</v>
       </c>
       <c r="J18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2017-22 CIC Pkg Loss Runs.PDF</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>openai/gpt-5.6-luna</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>21</v>
+      </c>
+      <c r="E19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="G19" t="n">
+        <v>19</v>
+      </c>
+      <c r="H19" t="n">
+        <v>12</v>
+      </c>
+      <c r="I19" t="n">
+        <v>63.2</v>
+      </c>
+      <c r="J19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -836,7 +872,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C2" t="n">
         <v>0</v>
@@ -868,13 +904,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D4" t="n">
-        <v>50</v>
+        <v>52.9</v>
       </c>
     </row>
     <row r="5">
@@ -884,13 +920,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C5" t="n">
         <v>10</v>
       </c>
       <c r="D5" t="n">
-        <v>62.5</v>
+        <v>58.8</v>
       </c>
     </row>
     <row r="6">
@@ -900,13 +936,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C6" t="n">
         <v>12</v>
       </c>
       <c r="D6" t="n">
-        <v>75</v>
+        <v>70.59999999999999</v>
       </c>
     </row>
     <row r="7">
@@ -916,13 +952,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C7" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D7" t="n">
-        <v>78.59999999999999</v>
+        <v>80</v>
       </c>
     </row>
     <row r="8">
@@ -932,90 +968,90 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C8" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D8" t="n">
-        <v>81.2</v>
+        <v>82.40000000000001</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Claim Number</t>
+          <t>Claim Status</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C9" t="n">
         <v>16</v>
       </c>
       <c r="D9" t="n">
-        <v>100</v>
+        <v>94.09999999999999</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Accident Date</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C10" t="n">
         <v>16</v>
       </c>
       <c r="D10" t="n">
-        <v>100</v>
+        <v>94.09999999999999</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Claim Status</t>
+          <t>Policy Number</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C11" t="n">
         <v>16</v>
       </c>
       <c r="D11" t="n">
-        <v>100</v>
+        <v>94.09999999999999</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Accident Date</t>
+          <t>Valuation Date</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C12" t="n">
         <v>16</v>
       </c>
       <c r="D12" t="n">
-        <v>100</v>
+        <v>94.09999999999999</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Report Date</t>
+          <t>Claim Number</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="C13" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="D13" t="n">
         <v>100</v>
@@ -1024,14 +1060,14 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Closed Date</t>
+          <t>Description</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C14" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D14" t="n">
         <v>100</v>
@@ -1040,7 +1076,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Loss State</t>
+          <t>Report Date</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1056,14 +1092,14 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Policy Number</t>
+          <t>Closed Date</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C16" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D16" t="n">
         <v>100</v>
@@ -1072,7 +1108,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Indemnity Paid</t>
+          <t>Loss State</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1088,14 +1124,14 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Indemnity Reserve</t>
+          <t>Indemnity Paid</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C18" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D18" t="n">
         <v>100</v>
@@ -1104,14 +1140,14 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Expense Paid</t>
+          <t>Indemnity Reserve</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C19" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D19" t="n">
         <v>100</v>
@@ -1120,14 +1156,14 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Expense Reserved</t>
+          <t>Expense Paid</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D20" t="n">
         <v>100</v>
@@ -1136,14 +1172,14 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Recovery Salvage Subro Reins</t>
+          <t>Expense Reserved</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C21" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D21" t="n">
         <v>100</v>
@@ -1152,14 +1188,14 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Recovery Deductible</t>
+          <t>Recovery Salvage Subro Reins</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C22" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D22" t="n">
         <v>100</v>
@@ -1168,14 +1204,14 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Valuation Date</t>
+          <t>Recovery Deductible</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="C23" t="n">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="D23" t="n">
         <v>100</v>
@@ -1188,10 +1224,10 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C24" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D24" t="n">
         <v>100</v>
@@ -1204,10 +1240,10 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C25" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D25" t="n">
         <v>100</v>
@@ -1314,28 +1350,28 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>18</v>
+        <v>39</v>
       </c>
       <c r="E2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G2" t="n">
-        <v>268</v>
+        <v>287</v>
       </c>
       <c r="H2" t="n">
-        <v>280</v>
+        <v>299</v>
       </c>
       <c r="I2" t="n">
-        <v>86.59999999999999</v>
+        <v>85</v>
       </c>
       <c r="J2" t="n">
-        <v>82.90000000000001</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="K2" t="n">
-        <v>3.7</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="3">
@@ -1355,28 +1391,28 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>18</v>
+        <v>39</v>
       </c>
       <c r="E3" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F3" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G3" t="n">
-        <v>268</v>
+        <v>287</v>
       </c>
       <c r="H3" t="n">
-        <v>268</v>
+        <v>287</v>
       </c>
       <c r="I3" t="n">
-        <v>86.59999999999999</v>
+        <v>85</v>
       </c>
       <c r="J3" t="n">
-        <v>86.59999999999999</v>
+        <v>84</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -1396,25 +1432,25 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>18</v>
+        <v>39</v>
       </c>
       <c r="E4" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F4" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G4" t="n">
-        <v>268</v>
+        <v>287</v>
       </c>
       <c r="H4" t="n">
-        <v>268</v>
+        <v>287</v>
       </c>
       <c r="I4" t="n">
-        <v>86.59999999999999</v>
+        <v>85</v>
       </c>
       <c r="J4" t="n">
-        <v>86.59999999999999</v>
+        <v>85</v>
       </c>
       <c r="K4" t="n">
         <v>0</v>
@@ -1437,25 +1473,25 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>18</v>
+        <v>39</v>
       </c>
       <c r="E5" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F5" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G5" t="n">
-        <v>268</v>
+        <v>287</v>
       </c>
       <c r="H5" t="n">
-        <v>268</v>
+        <v>287</v>
       </c>
       <c r="I5" t="n">
-        <v>86.59999999999999</v>
+        <v>85</v>
       </c>
       <c r="J5" t="n">
-        <v>86.59999999999999</v>
+        <v>85</v>
       </c>
       <c r="K5" t="n">
         <v>0</v>
@@ -1478,25 +1514,25 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>18</v>
+        <v>39</v>
       </c>
       <c r="E6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G6" t="n">
-        <v>268</v>
+        <v>287</v>
       </c>
       <c r="H6" t="n">
-        <v>268</v>
+        <v>287</v>
       </c>
       <c r="I6" t="n">
-        <v>86.59999999999999</v>
+        <v>85</v>
       </c>
       <c r="J6" t="n">
-        <v>86.59999999999999</v>
+        <v>85</v>
       </c>
       <c r="K6" t="n">
         <v>0</v>
@@ -1519,25 +1555,25 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>18</v>
+        <v>39</v>
       </c>
       <c r="E7" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F7" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G7" t="n">
-        <v>268</v>
+        <v>287</v>
       </c>
       <c r="H7" t="n">
-        <v>268</v>
+        <v>287</v>
       </c>
       <c r="I7" t="n">
-        <v>86.59999999999999</v>
+        <v>85</v>
       </c>
       <c r="J7" t="n">
-        <v>85.8</v>
+        <v>84.3</v>
       </c>
       <c r="K7" t="n">
         <v>0.7</v>
@@ -1639,7 +1675,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V23"/>
+  <dimension ref="A1:V28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1662,8 +1698,8 @@
     <col width="26" customWidth="1" min="18" max="18"/>
     <col width="26" customWidth="1" min="19" max="19"/>
     <col width="29" customWidth="1" min="20" max="20"/>
-    <col width="15" customWidth="1" min="21" max="21"/>
-    <col width="15" customWidth="1" min="22" max="22"/>
+    <col width="23" customWidth="1" min="21" max="21"/>
+    <col width="62" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2158,199 +2194,194 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7"/>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>5185622e</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>5abcb8d6104e</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2026-08-07 20:57:19</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2017-22 CIC Pkg Loss Runs.PDF</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>openai/gpt-5.6-luna</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>max</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>21</v>
+      </c>
+      <c r="I7" t="n">
+        <v>16</v>
+      </c>
+      <c r="J7" t="n">
+        <v>1</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="N7" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="O7" t="n">
+        <v>19</v>
+      </c>
+      <c r="P7" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>63.2</v>
+      </c>
+      <c r="R7" t="n">
+        <v>63.2</v>
+      </c>
+      <c r="S7" t="n">
+        <v>3</v>
+      </c>
+      <c r="T7" t="n">
+        <v>0</v>
+      </c>
+      <c r="U7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8"/>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>run_id</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>document</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>stage</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>model</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>provider</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>label</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>pages</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>attempt</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>effort</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>response_id</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>latency_s</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>poll_count</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>input_tokens</t>
         </is>
       </c>
-      <c r="O8" s="2" t="inlineStr">
+      <c r="O9" s="2" t="inlineStr">
         <is>
           <t>output_tokens</t>
         </is>
       </c>
-      <c r="P8" s="2" t="inlineStr">
+      <c r="P9" s="2" t="inlineStr">
         <is>
           <t>total_tokens</t>
         </is>
       </c>
-      <c r="Q8" s="2" t="inlineStr">
+      <c r="Q9" s="2" t="inlineStr">
         <is>
           <t>cost_input_usd</t>
         </is>
       </c>
-      <c r="R8" s="2" t="inlineStr">
+      <c r="R9" s="2" t="inlineStr">
         <is>
           <t>cost_output_usd</t>
         </is>
       </c>
-      <c r="S8" s="2" t="inlineStr">
+      <c r="S9" s="2" t="inlineStr">
         <is>
           <t>cost_total_usd</t>
         </is>
       </c>
-      <c r="T8" s="2" t="inlineStr">
+      <c r="T9" s="2" t="inlineStr">
         <is>
           <t>usage_missing</t>
         </is>
       </c>
-      <c r="U8" s="2" t="inlineStr">
+      <c r="U9" s="2" t="inlineStr">
         <is>
           <t>error_code</t>
         </is>
       </c>
-      <c r="V8" s="2" t="inlineStr">
+      <c r="V9" s="2" t="inlineStr">
         <is>
           <t>error_message</t>
         </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>40f183e1a55f</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>05.09.2020 to 6-30-2022- GL only Policy Loss Run Report.pdf</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>layout</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>openai/gpt-5.6-luna</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>openai</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>layout discovery</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>1-5</t>
-        </is>
-      </c>
-      <c r="H9" t="n">
-        <v>1</v>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>resp_0a4ea48cef7acdd3006a75f2ec13e4819393d541a8699901d6</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>completed</t>
-        </is>
-      </c>
-      <c r="L9" t="n">
-        <v>19.07</v>
-      </c>
-      <c r="M9" t="n">
-        <v>4</v>
-      </c>
-      <c r="N9" t="n">
-        <v>20226</v>
-      </c>
-      <c r="O9" t="n">
-        <v>1349</v>
-      </c>
-      <c r="P9" t="n">
-        <v>21575</v>
-      </c>
-      <c r="Q9" t="n">
-        <v>0.004045</v>
-      </c>
-      <c r="R9" t="n">
-        <v>0.001079</v>
-      </c>
-      <c r="S9" t="n">
-        <v>0.005124</v>
-      </c>
-      <c r="T9" t="b">
-        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -2366,7 +2397,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>extract</t>
+          <t>layout</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -2381,12 +2412,12 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>chunk 1/1</t>
+          <t>layout discovery</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>1-10</t>
+          <t>1-5</t>
         </is>
       </c>
       <c r="H10" t="n">
@@ -2394,12 +2425,12 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>max</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>resp_08a100fa287cdf15006a75f2fbd2708190bd7a78a62d98e308</t>
+          <t>resp_0a4ea48cef7acdd3006a75f2ec13e4819393d541a8699901d6</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -2408,28 +2439,28 @@
         </is>
       </c>
       <c r="L10" t="n">
-        <v>18.55</v>
+        <v>19.07</v>
       </c>
       <c r="M10" t="n">
         <v>4</v>
       </c>
       <c r="N10" t="n">
-        <v>35968</v>
+        <v>20226</v>
       </c>
       <c r="O10" t="n">
-        <v>21734</v>
+        <v>1349</v>
       </c>
       <c r="P10" t="n">
-        <v>57702</v>
+        <v>21575</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.007194</v>
+        <v>0.004045</v>
       </c>
       <c r="R10" t="n">
-        <v>0.017387</v>
+        <v>0.001079</v>
       </c>
       <c r="S10" t="n">
-        <v>0.024581</v>
+        <v>0.005124</v>
       </c>
       <c r="T10" t="b">
         <v>0</v>
@@ -2448,7 +2479,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>qa</t>
+          <t>extract</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -2481,7 +2512,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>resp_03817eba275b785f006a75f5e9e57481968eb800249d5c5530</t>
+          <t>resp_08a100fa287cdf15006a75f2fbd2708190bd7a78a62d98e308</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -2490,28 +2521,28 @@
         </is>
       </c>
       <c r="L11" t="n">
-        <v>68.41</v>
+        <v>18.55</v>
       </c>
       <c r="M11" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="N11" t="n">
-        <v>38119</v>
+        <v>35968</v>
       </c>
       <c r="O11" t="n">
-        <v>7415</v>
+        <v>21734</v>
       </c>
       <c r="P11" t="n">
-        <v>45534</v>
+        <v>57702</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.007624</v>
+        <v>0.007194</v>
       </c>
       <c r="R11" t="n">
-        <v>0.005932</v>
+        <v>0.017387</v>
       </c>
       <c r="S11" t="n">
-        <v>0.013556</v>
+        <v>0.024581</v>
       </c>
       <c r="T11" t="b">
         <v>0</v>
@@ -2520,17 +2551,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1759b6f93b6b</t>
+          <t>40f183e1a55f</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>16-18 GL Loss Runs - Twenty Mile Acceptance.pdf</t>
+          <t>05.09.2020 to 6-30-2022- GL only Policy Loss Run Report.pdf</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>layout</t>
+          <t>qa</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -2545,12 +2576,12 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>layout discovery</t>
+          <t>chunk 1/1</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>1-2</t>
+          <t>1-10</t>
         </is>
       </c>
       <c r="H12" t="n">
@@ -2558,12 +2589,12 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>max</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>resp_00fb79eac91891a0006a75f62f921c8197be64661c1c6f20f0</t>
+          <t>resp_03817eba275b785f006a75f5e9e57481968eb800249d5c5530</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -2572,28 +2603,28 @@
         </is>
       </c>
       <c r="L12" t="n">
-        <v>19.56</v>
+        <v>68.41</v>
       </c>
       <c r="M12" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="N12" t="n">
-        <v>12042</v>
+        <v>38119</v>
       </c>
       <c r="O12" t="n">
-        <v>1452</v>
+        <v>7415</v>
       </c>
       <c r="P12" t="n">
-        <v>13494</v>
+        <v>45534</v>
       </c>
       <c r="Q12" t="n">
-        <v>0.002408</v>
+        <v>0.007624</v>
       </c>
       <c r="R12" t="n">
-        <v>0.001162</v>
+        <v>0.005932</v>
       </c>
       <c r="S12" t="n">
-        <v>0.00357</v>
+        <v>0.013556</v>
       </c>
       <c r="T12" t="b">
         <v>0</v>
@@ -2612,7 +2643,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>extract</t>
+          <t>layout</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -2627,7 +2658,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>chunk 1/1</t>
+          <t>layout discovery</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -2640,12 +2671,12 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>max</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>resp_0752f25ff5cc747d006a75f642fe908196bf92abb84f96a388</t>
+          <t>resp_00fb79eac91891a0006a75f62f921c8197be64661c1c6f20f0</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -2654,28 +2685,28 @@
         </is>
       </c>
       <c r="L13" t="n">
-        <v>44.8</v>
+        <v>19.56</v>
       </c>
       <c r="M13" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="N13" t="n">
-        <v>12490</v>
+        <v>12042</v>
       </c>
       <c r="O13" t="n">
-        <v>5763</v>
+        <v>1452</v>
       </c>
       <c r="P13" t="n">
-        <v>18253</v>
+        <v>13494</v>
       </c>
       <c r="Q13" t="n">
-        <v>0.002498</v>
+        <v>0.002408</v>
       </c>
       <c r="R13" t="n">
-        <v>0.00461</v>
+        <v>0.001162</v>
       </c>
       <c r="S13" t="n">
-        <v>0.007108</v>
+        <v>0.00357</v>
       </c>
       <c r="T13" t="b">
         <v>0</v>
@@ -2694,7 +2725,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>qa</t>
+          <t>extract</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -2727,7 +2758,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>resp_01d001704000e301006a75f66f9edc81958828c4f26587423d</t>
+          <t>resp_0752f25ff5cc747d006a75f642fe908196bf92abb84f96a388</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -2736,28 +2767,28 @@
         </is>
       </c>
       <c r="L14" t="n">
-        <v>59.56</v>
+        <v>44.8</v>
       </c>
       <c r="M14" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="N14" t="n">
-        <v>13093</v>
+        <v>12490</v>
       </c>
       <c r="O14" t="n">
-        <v>6964</v>
+        <v>5763</v>
       </c>
       <c r="P14" t="n">
-        <v>20057</v>
+        <v>18253</v>
       </c>
       <c r="Q14" t="n">
-        <v>0.002619</v>
+        <v>0.002498</v>
       </c>
       <c r="R14" t="n">
-        <v>0.005571</v>
+        <v>0.00461</v>
       </c>
       <c r="S14" t="n">
-        <v>0.008189999999999999</v>
+        <v>0.007108</v>
       </c>
       <c r="T14" t="b">
         <v>0</v>
@@ -2766,17 +2797,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ccf6dacf0369</t>
+          <t>1759b6f93b6b</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>17-18 XS Loss Runs - AIG.pdf</t>
+          <t>16-18 GL Loss Runs - Twenty Mile Acceptance.pdf</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>layout</t>
+          <t>qa</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -2791,7 +2822,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>layout discovery</t>
+          <t>chunk 1/1</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -2804,12 +2835,12 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>max</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>resp_08e02d502f20a249006a75f6ad54bc819597d747c0721b717d</t>
+          <t>resp_01d001704000e301006a75f66f9edc81958828c4f26587423d</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -2818,28 +2849,28 @@
         </is>
       </c>
       <c r="L15" t="n">
-        <v>24</v>
+        <v>59.56</v>
       </c>
       <c r="M15" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="N15" t="n">
-        <v>9668</v>
+        <v>13093</v>
       </c>
       <c r="O15" t="n">
-        <v>1895</v>
+        <v>6964</v>
       </c>
       <c r="P15" t="n">
-        <v>11563</v>
+        <v>20057</v>
       </c>
       <c r="Q15" t="n">
-        <v>0.001934</v>
+        <v>0.002619</v>
       </c>
       <c r="R15" t="n">
-        <v>0.001516</v>
+        <v>0.005571</v>
       </c>
       <c r="S15" t="n">
-        <v>0.00345</v>
+        <v>0.008189999999999999</v>
       </c>
       <c r="T15" t="b">
         <v>0</v>
@@ -2858,7 +2889,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>extract</t>
+          <t>layout</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -2873,7 +2904,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>chunk 1/1</t>
+          <t>layout discovery</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -2886,12 +2917,12 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>max</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>resp_03005e22cdeeb03c006a75f6c5118c8195a40866eb7979f3d3</t>
+          <t>resp_08e02d502f20a249006a75f6ad54bc819597d747c0721b717d</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -2900,28 +2931,28 @@
         </is>
       </c>
       <c r="L16" t="n">
-        <v>103.07</v>
+        <v>24</v>
       </c>
       <c r="M16" t="n">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="N16" t="n">
-        <v>10034</v>
+        <v>9668</v>
       </c>
       <c r="O16" t="n">
-        <v>13255</v>
+        <v>1895</v>
       </c>
       <c r="P16" t="n">
-        <v>23289</v>
+        <v>11563</v>
       </c>
       <c r="Q16" t="n">
-        <v>0.002007</v>
+        <v>0.001934</v>
       </c>
       <c r="R16" t="n">
-        <v>0.010604</v>
+        <v>0.001516</v>
       </c>
       <c r="S16" t="n">
-        <v>0.012611</v>
+        <v>0.00345</v>
       </c>
       <c r="T16" t="b">
         <v>0</v>
@@ -2940,7 +2971,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>qa</t>
+          <t>extract</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -2973,7 +3004,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>resp_0a2bcc8f490832f6006a75f72c17dc8195ab8e88d1bb16c34b</t>
+          <t>resp_03005e22cdeeb03c006a75f6c5118c8195a40866eb7979f3d3</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -2982,28 +3013,28 @@
         </is>
       </c>
       <c r="L17" t="n">
-        <v>138.92</v>
+        <v>103.07</v>
       </c>
       <c r="M17" t="n">
-        <v>37</v>
+        <v>26</v>
       </c>
       <c r="N17" t="n">
-        <v>10309</v>
+        <v>10034</v>
       </c>
       <c r="O17" t="n">
-        <v>23380</v>
+        <v>13255</v>
       </c>
       <c r="P17" t="n">
-        <v>33689</v>
+        <v>23289</v>
       </c>
       <c r="Q17" t="n">
-        <v>0.002062</v>
+        <v>0.002007</v>
       </c>
       <c r="R17" t="n">
-        <v>0.018704</v>
+        <v>0.010604</v>
       </c>
       <c r="S17" t="n">
-        <v>0.020766</v>
+        <v>0.012611</v>
       </c>
       <c r="T17" t="b">
         <v>0</v>
@@ -3012,17 +3043,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>196521831d58</t>
+          <t>ccf6dacf0369</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>18-19 GL Loss Run - United Specialty.pdf</t>
+          <t>17-18 XS Loss Runs - AIG.pdf</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>layout</t>
+          <t>qa</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -3037,12 +3068,12 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>layout discovery</t>
+          <t>chunk 1/1</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>1-1</t>
+          <t>1-2</t>
         </is>
       </c>
       <c r="H18" t="n">
@@ -3050,12 +3081,12 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>max</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>resp_07524a2d2b102f7f006a75f7f4ca1881909daf67de0228efe6</t>
+          <t>resp_0a2bcc8f490832f6006a75f72c17dc8195ab8e88d1bb16c34b</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -3064,28 +3095,28 @@
         </is>
       </c>
       <c r="L18" t="n">
-        <v>16.31</v>
+        <v>138.92</v>
       </c>
       <c r="M18" t="n">
-        <v>4</v>
+        <v>37</v>
       </c>
       <c r="N18" t="n">
-        <v>8261</v>
+        <v>10309</v>
       </c>
       <c r="O18" t="n">
-        <v>1393</v>
+        <v>23380</v>
       </c>
       <c r="P18" t="n">
-        <v>9654</v>
+        <v>33689</v>
       </c>
       <c r="Q18" t="n">
-        <v>0.001652</v>
+        <v>0.002062</v>
       </c>
       <c r="R18" t="n">
-        <v>0.001114</v>
+        <v>0.018704</v>
       </c>
       <c r="S18" t="n">
-        <v>0.002767</v>
+        <v>0.020766</v>
       </c>
       <c r="T18" t="b">
         <v>0</v>
@@ -3104,7 +3135,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>extract</t>
+          <t>layout</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -3119,7 +3150,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>chunk 1/1</t>
+          <t>layout discovery</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -3132,12 +3163,12 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>max</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>resp_0ecd97c337817288006a75f804d5ac8190a98cec5129c5f380</t>
+          <t>resp_07524a2d2b102f7f006a75f7f4ca1881909daf67de0228efe6</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -3146,28 +3177,28 @@
         </is>
       </c>
       <c r="L19" t="n">
-        <v>22.74</v>
+        <v>16.31</v>
       </c>
       <c r="M19" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="N19" t="n">
-        <v>8651</v>
+        <v>8261</v>
       </c>
       <c r="O19" t="n">
-        <v>2575</v>
+        <v>1393</v>
       </c>
       <c r="P19" t="n">
-        <v>11226</v>
+        <v>9654</v>
       </c>
       <c r="Q19" t="n">
-        <v>0.00173</v>
+        <v>0.001652</v>
       </c>
       <c r="R19" t="n">
-        <v>0.00206</v>
+        <v>0.001114</v>
       </c>
       <c r="S19" t="n">
-        <v>0.00379</v>
+        <v>0.002767</v>
       </c>
       <c r="T19" t="b">
         <v>0</v>
@@ -3186,7 +3217,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>qa</t>
+          <t>extract</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -3219,7 +3250,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>resp_04ffca1fcc2e0ecc006a75f81b8ea88193a1aa1ce03f5ac990</t>
+          <t>resp_0ecd97c337817288006a75f804d5ac8190a98cec5129c5f380</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -3228,28 +3259,28 @@
         </is>
       </c>
       <c r="L20" t="n">
-        <v>34.13</v>
+        <v>22.74</v>
       </c>
       <c r="M20" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="N20" t="n">
-        <v>8902</v>
+        <v>8651</v>
       </c>
       <c r="O20" t="n">
-        <v>3536</v>
+        <v>2575</v>
       </c>
       <c r="P20" t="n">
-        <v>12438</v>
+        <v>11226</v>
       </c>
       <c r="Q20" t="n">
-        <v>0.00178</v>
+        <v>0.00173</v>
       </c>
       <c r="R20" t="n">
-        <v>0.002829</v>
+        <v>0.00206</v>
       </c>
       <c r="S20" t="n">
-        <v>0.004609</v>
+        <v>0.00379</v>
       </c>
       <c r="T20" t="b">
         <v>0</v>
@@ -3258,17 +3289,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>3e0fb97b3ce7</t>
+          <t>196521831d58</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>18-19 XS Loss Runs - AIG.pdf</t>
+          <t>18-19 GL Loss Run - United Specialty.pdf</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>layout</t>
+          <t>qa</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -3283,7 +3314,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>layout discovery</t>
+          <t>chunk 1/1</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -3296,12 +3327,12 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>max</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>resp_029cf6536e8ff7b5006a75f84167c481949dd80cb7ea79b942</t>
+          <t>resp_04ffca1fcc2e0ecc006a75f81b8ea88193a1aa1ce03f5ac990</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -3310,28 +3341,28 @@
         </is>
       </c>
       <c r="L21" t="n">
-        <v>23.57</v>
+        <v>34.13</v>
       </c>
       <c r="M21" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="N21" t="n">
-        <v>7368</v>
+        <v>8902</v>
       </c>
       <c r="O21" t="n">
-        <v>1851</v>
+        <v>3536</v>
       </c>
       <c r="P21" t="n">
-        <v>9219</v>
+        <v>12438</v>
       </c>
       <c r="Q21" t="n">
-        <v>0.001474</v>
+        <v>0.00178</v>
       </c>
       <c r="R21" t="n">
-        <v>0.001481</v>
+        <v>0.002829</v>
       </c>
       <c r="S21" t="n">
-        <v>0.002954</v>
+        <v>0.004609</v>
       </c>
       <c r="T21" t="b">
         <v>0</v>
@@ -3350,7 +3381,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>extract</t>
+          <t>layout</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -3365,7 +3396,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>chunk 1/1</t>
+          <t>layout discovery</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -3378,12 +3409,12 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>max</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>resp_0dbf9fdfbe24bcaf006a75f858be408196b5564146a5d5d081</t>
+          <t>resp_029cf6536e8ff7b5006a75f84167c481949dd80cb7ea79b942</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -3392,28 +3423,28 @@
         </is>
       </c>
       <c r="L22" t="n">
-        <v>103.6</v>
+        <v>23.57</v>
       </c>
       <c r="M22" t="n">
-        <v>28</v>
+        <v>6</v>
       </c>
       <c r="N22" t="n">
-        <v>7683</v>
+        <v>7368</v>
       </c>
       <c r="O22" t="n">
-        <v>13721</v>
+        <v>1851</v>
       </c>
       <c r="P22" t="n">
-        <v>21404</v>
+        <v>9219</v>
       </c>
       <c r="Q22" t="n">
-        <v>0.001537</v>
+        <v>0.001474</v>
       </c>
       <c r="R22" t="n">
-        <v>0.010977</v>
+        <v>0.001481</v>
       </c>
       <c r="S22" t="n">
-        <v>0.012513</v>
+        <v>0.002954</v>
       </c>
       <c r="T22" t="b">
         <v>0</v>
@@ -3432,72 +3463,487 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
+          <t>extract</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>openai/gpt-5.6-luna</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>openai</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>chunk 1/1</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H23" t="n">
+        <v>1</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>max</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>resp_0dbf9fdfbe24bcaf006a75f858be408196b5564146a5d5d081</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="L23" t="n">
+        <v>103.6</v>
+      </c>
+      <c r="M23" t="n">
+        <v>28</v>
+      </c>
+      <c r="N23" t="n">
+        <v>7683</v>
+      </c>
+      <c r="O23" t="n">
+        <v>13721</v>
+      </c>
+      <c r="P23" t="n">
+        <v>21404</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>0.001537</v>
+      </c>
+      <c r="R23" t="n">
+        <v>0.010977</v>
+      </c>
+      <c r="S23" t="n">
+        <v>0.012513</v>
+      </c>
+      <c r="T23" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>3e0fb97b3ce7</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>18-19 XS Loss Runs - AIG.pdf</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
           <t>qa</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>openai/gpt-5.6-luna</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>openai</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="F24" t="inlineStr">
         <is>
           <t>chunk 1/1</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="G24" t="inlineStr">
         <is>
           <t>1-1</t>
         </is>
       </c>
-      <c r="H23" t="n">
-        <v>1</v>
-      </c>
-      <c r="I23" t="inlineStr">
+      <c r="H24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I24" t="inlineStr">
         <is>
           <t>max</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
+      <c r="J24" t="inlineStr">
         <is>
           <t>resp_0c97261014dfacf8006a75f8c04fd88190addffbea021f4f99</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr">
+      <c r="K24" t="inlineStr">
         <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="L23" t="n">
+      <c r="L24" t="n">
         <v>131.5</v>
       </c>
-      <c r="M23" t="n">
+      <c r="M24" t="n">
         <v>35</v>
       </c>
-      <c r="N23" t="n">
+      <c r="N24" t="n">
         <v>7968</v>
       </c>
-      <c r="O23" t="n">
+      <c r="O24" t="n">
         <v>18533</v>
       </c>
-      <c r="P23" t="n">
+      <c r="P24" t="n">
         <v>26501</v>
       </c>
-      <c r="Q23" t="n">
+      <c r="Q24" t="n">
         <v>0.001594</v>
       </c>
-      <c r="R23" t="n">
+      <c r="R24" t="n">
         <v>0.014826</v>
       </c>
-      <c r="S23" t="n">
+      <c r="S24" t="n">
         <v>0.01642</v>
       </c>
-      <c r="T23" t="b">
+      <c r="T24" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>5abcb8d6104e</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2017-22 CIC Pkg Loss Runs.PDF</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>layout</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>openai/gpt-5.6-luna</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>openai</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>layout discovery</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H25" t="n">
+        <v>1</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>resp_0ca34eba266ba722006a75f958587c8196ae8f11772e4defe3</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="L25" t="n">
+        <v>22.53</v>
+      </c>
+      <c r="M25" t="n">
+        <v>6</v>
+      </c>
+      <c r="N25" t="n">
+        <v>13825</v>
+      </c>
+      <c r="O25" t="n">
+        <v>1946</v>
+      </c>
+      <c r="P25" t="n">
+        <v>15771</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>0.002765</v>
+      </c>
+      <c r="R25" t="n">
+        <v>0.001557</v>
+      </c>
+      <c r="S25" t="n">
+        <v>0.004322</v>
+      </c>
+      <c r="T25" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>5abcb8d6104e</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2017-22 CIC Pkg Loss Runs.PDF</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>extract</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>openai/gpt-5.6-luna</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>openai</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>chunk 1/1</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H26" t="n">
+        <v>1</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>max</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>resp_008f41fab534903c006a75f96ed29c81959239f015ea24c390</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="L26" t="n">
+        <v>150.23</v>
+      </c>
+      <c r="M26" t="n">
+        <v>40</v>
+      </c>
+      <c r="N26" t="n">
+        <v>14244</v>
+      </c>
+      <c r="O26" t="n">
+        <v>28585</v>
+      </c>
+      <c r="P26" t="n">
+        <v>42829</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>0.002849</v>
+      </c>
+      <c r="R26" t="n">
+        <v>0.022868</v>
+      </c>
+      <c r="S26" t="n">
+        <v>0.025717</v>
+      </c>
+      <c r="T26" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>5abcb8d6104e</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2017-22 CIC Pkg Loss Runs.PDF</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>qa</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>openai/gpt-5.6-luna</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>openai</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>chunk 1/1</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H27" t="n">
+        <v>1</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>max</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="L27" t="n">
+        <v>104.07</v>
+      </c>
+      <c r="M27" t="n">
+        <v>0</v>
+      </c>
+      <c r="N27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O27" t="n">
+        <v>0</v>
+      </c>
+      <c r="P27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>0</v>
+      </c>
+      <c r="R27" t="n">
+        <v>0</v>
+      </c>
+      <c r="S27" t="n">
+        <v>0</v>
+      </c>
+      <c r="T27" t="b">
+        <v>0</v>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>invalid_request_error</t>
+        </is>
+      </c>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>HTTP 404: Response with id 'resp_02bd3292dc08c691006a75fb87ede48193944af1e703bea915' not found.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>5abcb8d6104e</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2017-22 CIC Pkg Loss Runs.PDF</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>qa</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>openai/gpt-5.6-luna</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>openai</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>chunk 1/1</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H28" t="n">
+        <v>2</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>max</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>resp_0a0873450ce8a4cc006a760cc147f88197b8649a90a483f714</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="L28" t="n">
+        <v>279.01</v>
+      </c>
+      <c r="M28" t="n">
+        <v>46</v>
+      </c>
+      <c r="N28" t="n">
+        <v>16069</v>
+      </c>
+      <c r="O28" t="n">
+        <v>29536</v>
+      </c>
+      <c r="P28" t="n">
+        <v>45605</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>0.003214</v>
+      </c>
+      <c r="R28" t="n">
+        <v>0.023629</v>
+      </c>
+      <c r="S28" t="n">
+        <v>0.026843</v>
+      </c>
+      <c r="T28" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>